<commit_message>
Add success message validation and refactor ContactPage
</commit_message>
<xml_diff>
--- a/src/test/resources/massa/Massa/automationExercise.xlsx
+++ b/src/test/resources/massa/Massa/automationExercise.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="15">
   <si>
     <t>CT</t>
   </si>
@@ -19,10 +19,10 @@
     <t>EMAIL</t>
   </si>
   <si>
-    <t>SENHA</t>
+    <t xml:space="preserve">PASSWORD </t>
   </si>
   <si>
-    <t>NOME</t>
+    <t>NAME</t>
   </si>
   <si>
     <t>SUBJECT</t>
@@ -40,6 +40,12 @@
     <t>asdf1234</t>
   </si>
   <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEST AUTOMATION </t>
+  </si>
+  <si>
     <t>2</t>
   </si>
   <si>
@@ -50,18 +56,6 @@
   </si>
   <si>
     <t>4</t>
-  </si>
-  <si>
-    <t>TEST</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TESTINHO </t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEST AUTOMATION </t>
   </si>
 </sst>
 </file>
@@ -133,11 +127,11 @@
     <xf quotePrefix="1" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
+    <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0"/>
+    </xf>
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf quotePrefix="1" borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center"/>
@@ -416,9 +410,15 @@
       <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="5"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>10</v>
+      </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
@@ -442,7 +442,7 @@
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>7</v>
@@ -450,7 +450,7 @@
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="5"/>
+      <c r="D3" s="6"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -479,12 +479,12 @@
         <v>3.0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
-      <c r="D4" s="5"/>
+      <c r="D4" s="6"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -510,14 +510,14 @@
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="5"/>
+      <c r="C5" s="6"/>
       <c r="D5" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
@@ -543,22 +543,12 @@
       <c r="Z5" s="3"/>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="A6" s="7"/>
+      <c r="B6" s="3"/>
       <c r="C6" s="3"/>
-      <c r="D6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>16</v>
-      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -581,11 +571,11 @@
       <c r="Z6" s="3"/>
     </row>
     <row r="7">
-      <c r="A7" s="7"/>
+      <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
+      <c r="E7" s="7"/>
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
@@ -725,7 +715,7 @@
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
+      <c r="E12" s="7"/>
       <c r="F12" s="3"/>
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
@@ -752,8 +742,8 @@
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="3"/>
       <c r="F13" s="3"/>
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
@@ -1537,7 +1527,7 @@
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
+      <c r="E41" s="7"/>
       <c r="F41" s="3"/>
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
@@ -1565,7 +1555,7 @@
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
       <c r="D42" s="3"/>
-      <c r="E42" s="7"/>
+      <c r="E42" s="3"/>
       <c r="F42" s="3"/>
       <c r="G42" s="3"/>
       <c r="H42" s="3"/>
@@ -28412,34 +28402,6 @@
       <c r="Y1000" s="3"/>
       <c r="Z1000" s="3"/>
     </row>
-    <row r="1001">
-      <c r="A1001" s="3"/>
-      <c r="B1001" s="3"/>
-      <c r="C1001" s="3"/>
-      <c r="D1001" s="3"/>
-      <c r="E1001" s="3"/>
-      <c r="F1001" s="3"/>
-      <c r="G1001" s="3"/>
-      <c r="H1001" s="3"/>
-      <c r="I1001" s="3"/>
-      <c r="J1001" s="3"/>
-      <c r="K1001" s="3"/>
-      <c r="L1001" s="3"/>
-      <c r="M1001" s="3"/>
-      <c r="N1001" s="3"/>
-      <c r="O1001" s="3"/>
-      <c r="P1001" s="3"/>
-      <c r="Q1001" s="3"/>
-      <c r="R1001" s="3"/>
-      <c r="S1001" s="3"/>
-      <c r="T1001" s="3"/>
-      <c r="U1001" s="3"/>
-      <c r="V1001" s="3"/>
-      <c r="W1001" s="3"/>
-      <c r="X1001" s="3"/>
-      <c r="Y1001" s="3"/>
-      <c r="Z1001" s="3"/>
-    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>